<commit_message>
Changed BOM Excel and removes wrong PCB geber
</commit_message>
<xml_diff>
--- a/v1/JLCPCB Order/Bill of Materials.xlsx
+++ b/v1/JLCPCB Order/Bill of Materials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Client\Documents\GitHub\rfid-nfc-manager\JLCPCB Order\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Client\Documents\GitHub\rfid-nfc-manager\v1\JLCPCB Order\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16BB713D-6689-4478-B8C2-7A038E6DEC2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D615B3-288C-4C8E-9DDB-945AED9B87D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15480" xr2:uid="{33F2DA52-EEA3-47B3-A567-6D5168423C5F}"/>
+    <workbookView xWindow="25485" yWindow="0" windowWidth="13020" windowHeight="15285" xr2:uid="{33F2DA52-EEA3-47B3-A567-6D5168423C5F}"/>
   </bookViews>
   <sheets>
     <sheet name="RFID" sheetId="3" r:id="rId1"/>
@@ -181,9 +181,6 @@
     <t>https://www.mouser.pl/en/ProductDetail/Semtech/RCLAMP03331PWQC?qs=wT7LY0lnAe0Cyd1U%2FGqM7A%3D%3D</t>
   </si>
   <si>
-    <t>https://assets.nexperia.com/documents/data-sheet/PTVS5V0Z1USK.pdf</t>
-  </si>
-  <si>
     <t>F1</t>
   </si>
   <si>
@@ -752,6 +749,9 @@
   </si>
   <si>
     <t>https://www.mouser.pl/en/ProductDetail/Molex/15134-0301?qs=lQAVKuKFhkL4Aonld%2FWL2g%3D%3D</t>
+  </si>
+  <si>
+    <t>https://www.mouser.pl/en/ProductDetail/Wurth-Elektronik/824520600?qs=16w8nSHsg3vYKDXdaWEC1w%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -806,7 +806,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -820,6 +820,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -827,14 +828,14 @@
   </cellStyles>
   <dxfs count="6">
     <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;zł&quot;"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;zł&quot;"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;zł&quot;"/>
@@ -883,11 +884,11 @@
     <tableColumn id="3" xr3:uid="{0CE96DDB-24C8-4DA3-BADA-AE7896D3402B}" uniqueName="3" name="Value" queryTableFieldId="3" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{913BA5DE-D16C-49E5-BCC5-928AE6C6536C}" uniqueName="2" name="Qty" queryTableFieldId="2"/>
     <tableColumn id="6" xr3:uid="{5AA8CCA3-4938-44BC-86B7-1719F7D4981E}" uniqueName="6" name="Price" queryTableFieldId="6" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{009DB6CD-5A08-4ECD-8CC1-A6F04554B046}" uniqueName="7" name="Full Price" queryTableFieldId="7" dataDxfId="0">
+    <tableColumn id="7" xr3:uid="{009DB6CD-5A08-4ECD-8CC1-A6F04554B046}" uniqueName="7" name="Full Price" queryTableFieldId="7" dataDxfId="2">
       <calculatedColumnFormula>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{C5D5866C-93DB-43C2-906C-8763999F1784}" uniqueName="5" name="Name" queryTableFieldId="5" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{B3E4820C-7529-4EB8-8FDB-C30FFBA22F3F}" uniqueName="4" name="Site" queryTableFieldId="4" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C5D5866C-93DB-43C2-906C-8763999F1784}" uniqueName="5" name="Name" queryTableFieldId="5" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{B3E4820C-7529-4EB8-8FDB-C30FFBA22F3F}" uniqueName="4" name="Site" queryTableFieldId="4" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1233,16 +1234,16 @@
         <v>1</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="F1" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="G1" t="s">
         <v>184</v>
-      </c>
-      <c r="G1" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1263,7 +1264,7 @@
         <v>10.039999999999999</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>5</v>
@@ -1287,7 +1288,7 @@
         <v>1.8049999999999999</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>8</v>
@@ -1311,7 +1312,7 @@
         <v>1.5960000000000001</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>11</v>
@@ -1319,7 +1320,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B5" t="s">
         <v>12</v>
@@ -1335,7 +1336,7 @@
         <v>2.2050000000000001</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>13</v>
@@ -1359,10 +1360,10 @@
         <v>1.41</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1383,7 +1384,7 @@
         <v>1.08</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>18</v>
@@ -1407,7 +1408,7 @@
         <v>1.63</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>21</v>
@@ -1431,7 +1432,7 @@
         <v>1.302</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>24</v>
@@ -1455,7 +1456,7 @@
         <v>0.5</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>27</v>
@@ -1487,7 +1488,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -1502,7 +1503,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C13">
         <v>2</v>
@@ -1530,7 +1531,7 @@
         <v>2.16</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>35</v>
@@ -1554,7 +1555,7 @@
         <v>0.39900000000000002</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>38</v>
@@ -1565,7 +1566,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -1578,10 +1579,10 @@
         <v>0.83199999999999996</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1589,7 +1590,7 @@
         <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C17">
         <v>3</v>
@@ -1602,7 +1603,7 @@
         <v>7.17</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>41</v>
@@ -1610,10 +1611,10 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B18" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C18">
         <v>2</v>
@@ -1629,15 +1630,15 @@
         <v>824520600</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>42</v>
+        <v>232</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B19" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1650,42 +1651,42 @@
         <v>1.1599999999999999</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" t="s">
         <v>45</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E20" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="G20" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-      <c r="D20" s="6">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E20" s="3">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C21">
         <v>2</v>
@@ -1698,18 +1699,18 @@
         <v>0.72199999999999998</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B22" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C22">
         <v>5</v>
@@ -1722,18 +1723,18 @@
         <v>7.8900000000000006</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B23" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C23">
         <v>5</v>
@@ -1746,18 +1747,18 @@
         <v>32.99</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -1770,18 +1771,18 @@
         <v>12.39</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B25" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -1794,18 +1795,18 @@
         <v>4.45</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B26" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -1818,18 +1819,18 @@
         <v>1.63</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>192</v>
+      </c>
+      <c r="B27" t="s">
         <v>193</v>
-      </c>
-      <c r="B27" t="s">
-        <v>194</v>
       </c>
       <c r="C27">
         <v>3</v>
@@ -1842,18 +1843,18 @@
         <v>4.32</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B28" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -1866,15 +1867,15 @@
         <v>1.7</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B29" t="s">
         <v>7</v>
@@ -1890,18 +1891,18 @@
         <v>0.90300000000000002</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" t="s">
         <v>61</v>
-      </c>
-      <c r="B30" t="s">
-        <v>62</v>
       </c>
       <c r="C30">
         <v>2</v>
@@ -1914,18 +1915,18 @@
         <v>1.444</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" t="s">
         <v>65</v>
-      </c>
-      <c r="B31" t="s">
-        <v>66</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -1938,18 +1939,18 @@
         <v>1.44</v>
       </c>
       <c r="F31" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="G31" s="1" t="s">
         <v>208</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B32" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1962,18 +1963,18 @@
         <v>0.72199999999999998</v>
       </c>
       <c r="F32" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G32" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B33" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -1986,66 +1987,66 @@
         <v>0.504</v>
       </c>
       <c r="F33" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G33" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B34" t="s">
+        <v>211</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E34" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="C34">
-        <v>1</v>
-      </c>
-      <c r="D34" s="6">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E34" s="3">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>73</v>
+      </c>
+      <c r="B35" t="s">
         <v>74</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E35" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G35" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="C35">
-        <v>1</v>
-      </c>
-      <c r="D35" s="6">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E35" s="3">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>77</v>
+      </c>
+      <c r="B36" t="s">
         <v>78</v>
-      </c>
-      <c r="B36" t="s">
-        <v>79</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -2058,90 +2059,90 @@
         <v>0.45400000000000001</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>80</v>
+      </c>
+      <c r="B37" t="s">
         <v>81</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37">
+        <v>1</v>
+      </c>
+      <c r="D37" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E37" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="G37" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="C37">
-        <v>1</v>
-      </c>
-      <c r="D37" s="6">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E37" s="3">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>83</v>
+      </c>
+      <c r="B38" t="s">
         <v>84</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E38" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="G38" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="C38">
-        <v>1</v>
-      </c>
-      <c r="D38" s="6">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E38" s="3">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>87</v>
+      </c>
+      <c r="B39" t="s">
         <v>88</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E39" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="G39" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C39">
-        <v>1</v>
-      </c>
-      <c r="D39" s="6">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E39" s="3">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>91</v>
+      </c>
+      <c r="B40" t="s">
         <v>92</v>
-      </c>
-      <c r="B40" t="s">
-        <v>93</v>
       </c>
       <c r="C40">
         <v>2</v>
@@ -2154,18 +2155,18 @@
         <v>0.72199999999999998</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>94</v>
+      </c>
+      <c r="B41" t="s">
         <v>95</v>
-      </c>
-      <c r="B41" t="s">
-        <v>96</v>
       </c>
       <c r="C41">
         <v>2</v>
@@ -2178,18 +2179,18 @@
         <v>0.72199999999999998</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>97</v>
+      </c>
+      <c r="B42" t="s">
         <v>98</v>
-      </c>
-      <c r="B42" t="s">
-        <v>99</v>
       </c>
       <c r="C42">
         <v>5</v>
@@ -2202,67 +2203,67 @@
         <v>1.8049999999999999</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>100</v>
+      </c>
+      <c r="B43" t="s">
+        <v>81</v>
+      </c>
+      <c r="C43">
+        <v>1</v>
+      </c>
+      <c r="D43" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E43" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="G43" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="B43" t="s">
-        <v>82</v>
-      </c>
-      <c r="C43">
-        <v>1</v>
-      </c>
-      <c r="D43" s="6">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E43" s="3">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F43" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>102</v>
+      </c>
+      <c r="B44" t="s">
         <v>103</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44">
+        <v>1</v>
+      </c>
+      <c r="D44" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E44" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="G44" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="C44">
-        <v>1</v>
-      </c>
-      <c r="D44" s="6">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E44" s="3">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>105</v>
+      </c>
+      <c r="B45" t="s">
         <v>106</v>
       </c>
-      <c r="B45" t="s">
-        <v>107</v>
-      </c>
       <c r="C45">
         <v>1</v>
       </c>
@@ -2274,39 +2275,39 @@
         <v>0.36099999999999999</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>107</v>
+      </c>
+      <c r="B46" t="s">
         <v>108</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46">
+        <v>1</v>
+      </c>
+      <c r="D46" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E46" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="G46" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="C46">
-        <v>1</v>
-      </c>
-      <c r="D46" s="6">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E46" s="3">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F46" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C47">
         <v>2</v>
@@ -2320,10 +2321,10 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>110</v>
+      </c>
+      <c r="B48" t="s">
         <v>111</v>
-      </c>
-      <c r="B48" t="s">
-        <v>112</v>
       </c>
       <c r="C48">
         <v>2</v>
@@ -2336,66 +2337,66 @@
         <v>0.72199999999999998</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>113</v>
+      </c>
+      <c r="B49" t="s">
+        <v>95</v>
+      </c>
+      <c r="C49">
+        <v>1</v>
+      </c>
+      <c r="D49" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E49" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="G49" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B49" t="s">
-        <v>96</v>
-      </c>
-      <c r="C49">
-        <v>1</v>
-      </c>
-      <c r="D49" s="6">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E49" s="3">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F49" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>115</v>
+      </c>
+      <c r="B50" t="s">
         <v>116</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50">
+        <v>1</v>
+      </c>
+      <c r="D50" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E50" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="G50" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="C50">
-        <v>1</v>
-      </c>
-      <c r="D50" s="6">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E50" s="3">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B51" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C51">
         <v>4</v>
@@ -2408,18 +2409,18 @@
         <v>1.444</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>121</v>
+      </c>
+      <c r="B52" t="s">
         <v>122</v>
-      </c>
-      <c r="B52" t="s">
-        <v>123</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -2432,18 +2433,18 @@
         <v>0.45400000000000001</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>124</v>
+      </c>
+      <c r="B53" t="s">
         <v>125</v>
-      </c>
-      <c r="B53" t="s">
-        <v>126</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -2456,18 +2457,18 @@
         <v>3.68</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B54" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -2480,18 +2481,18 @@
         <v>1.73</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>163</v>
+      </c>
+      <c r="B55" t="s">
         <v>164</v>
-      </c>
-      <c r="B55" t="s">
-        <v>165</v>
       </c>
       <c r="C55">
         <v>2</v>
@@ -2504,18 +2505,18 @@
         <v>1.0840000000000001</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>165</v>
+      </c>
+      <c r="B56" t="s">
         <v>166</v>
-      </c>
-      <c r="B56" t="s">
-        <v>167</v>
       </c>
       <c r="C56">
         <v>2</v>
@@ -2528,18 +2529,18 @@
         <v>1.008</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B57" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C57">
         <v>1</v>
@@ -2552,18 +2553,18 @@
         <v>1.19</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B58" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -2576,18 +2577,18 @@
         <v>2.56</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B59" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C59">
         <v>1</v>
@@ -2600,18 +2601,18 @@
         <v>12.64</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>137</v>
+      </c>
+      <c r="B60" t="s">
         <v>138</v>
-      </c>
-      <c r="B60" t="s">
-        <v>139</v>
       </c>
       <c r="C60">
         <v>1</v>
@@ -2624,18 +2625,18 @@
         <v>4.01</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>140</v>
+      </c>
+      <c r="B61" t="s">
         <v>141</v>
-      </c>
-      <c r="B61" t="s">
-        <v>142</v>
       </c>
       <c r="C61">
         <v>1</v>
@@ -2648,15 +2649,15 @@
         <v>2.13</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C62">
         <v>1</v>
@@ -2668,8 +2669,8 @@
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>11.8</v>
       </c>
-      <c r="G62" t="s">
-        <v>232</v>
+      <c r="G62" s="7" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
@@ -2739,10 +2740,11 @@
     <hyperlink ref="G61" r:id="rId55" xr:uid="{E3E03E0B-FDF9-44F6-BC71-51F037465404}"/>
     <hyperlink ref="G27" r:id="rId56" xr:uid="{8B5ED6F3-6A10-4B07-9C09-D15BA3C4B9B2}"/>
     <hyperlink ref="G34" r:id="rId57" xr:uid="{D7262D6F-B67E-4B7E-94F1-5ACE83FC45C3}"/>
+    <hyperlink ref="G62" r:id="rId58" xr:uid="{1EB70F93-9549-48EF-B11F-F7E056F6B2FA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId58"/>
+    <tablePart r:id="rId59"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>